<commit_message>
Reagrupar el catálogo ANS BD en 6 categorías por función (a prueba de futuro)
Las categorías dejan de nombrar artefactos específicos (plantillas de
contacto, material de entendimiento) y pasan a cajones por función:
Evidencia y diagnóstico, Comunicación conductual, Arquitectura de
intervención, Validación y experimentación, Sistemas y frameworks,
Adopción y despliegue. Cada una lista ejemplos actuales del Q3 y
futuros, con regla de encaje para quests que combinan funciones.
MD y Excel actualizados en el mismo formato visual de Milagros.
</commit_message>
<xml_diff>
--- a/reportes/ANS_Behavioral_Design_propuesta.xlsx
+++ b/reportes/ANS_Behavioral_Design_propuesta.xlsx
@@ -654,7 +654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -989,18 +989,18 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="20" t="inlineStr">
         <is>
-          <t>Material de entendimiento
-(guía resumida, flyer, carta — guías AMI, EPS)</t>
+          <t>🔍 Evidencia y diagnóstico
+(desk research, bench, behavioral journey, diagnóstico de barreras, análisis de data conductual)</t>
         </is>
       </c>
       <c r="B10" s="21" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="C10" s="21" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="D10" s="21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E10" s="21" t="n">
         <v>12</v>
@@ -1044,8 +1044,8 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="20" t="inlineStr">
         <is>
-          <t>Playbook / método
-(playbook de ventas, playbook B360)</t>
+          <t>📣 Comunicación conductual
+(guías resumidas, flyers, cartas, plantillas de mensaje para asesores, guías de comunicación con speeches, journeys, notificaciones)</t>
         </is>
       </c>
       <c r="B11" s="21" t="n">
@@ -1055,7 +1055,7 @@
         <v>3.5</v>
       </c>
       <c r="D11" s="21" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E11" s="21" t="n">
         <v>12</v>
@@ -1099,21 +1099,21 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>Estrategia + plantillas de contacto
-(informe CUA, plantillas WhatsApp/correo)</t>
+          <t>🎛️ Arquitectura de intervención
+(estrategia de primer contacto, defaults, rediseño de momentos de decisión, sistemas de incentivos)</t>
         </is>
       </c>
       <c r="B12" s="21" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="C12" s="21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D12" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E12" s="21" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F12" s="22">
         <f>B12*$F$4</f>
@@ -1154,21 +1154,21 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="20" t="inlineStr">
         <is>
-          <t>Diagnóstico conductual / research
-(desk research, bench frío/caliente)</t>
+          <t>🧪 Validación y experimentación
+(sacrificial concepts, tests de concepto, pilotos, experimentos A/B con tracking)</t>
         </is>
       </c>
       <c r="B13" s="21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C13" s="21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D13" s="21" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E13" s="21" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F13" s="22">
         <f>B13*$F$4</f>
@@ -1209,12 +1209,12 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>Test de concepto / experimento
-(Vivo Pack, sacrificial concepts)</t>
+          <t>📚 Sistemas y frameworks
+(playbooks, modelos de competencias/hábitos, bibliotecas de intervenciones, guidelines para otros equipos)</t>
         </is>
       </c>
       <c r="B14" s="21" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="C14" s="21" t="n">
         <v>5</v>
@@ -1264,28 +1264,25 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="20" t="inlineStr">
         <is>
-          <t>Modelo / framework
-(modelo de competencias, cambio de hábitos)</t>
-        </is>
-      </c>
-      <c r="B15" s="21" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+          <t>🚀 Adopción y despliegue
+(despliegues FFVV/UV, capacitaciones, campañas de adopción, seguimiento post-implementación)</t>
+        </is>
+      </c>
+      <c r="B15" s="21" t="n">
+        <v>1.5</v>
       </c>
       <c r="C15" s="21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D15" s="21" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E15" s="21" t="n">
-        <v>15</v>
-      </c>
-      <c r="F15" s="21" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>12</v>
+      </c>
+      <c r="F15" s="22">
+        <f>B15*$F$4</f>
+        <v/>
       </c>
       <c r="G15" s="22">
         <f>C15*$F$4</f>
@@ -1302,10 +1299,9 @@
       <c r="J15" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K15" s="21" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+      <c r="K15" s="21">
+        <f>B15+$J15</f>
+        <v/>
       </c>
       <c r="L15" s="21">
         <f>C15+$J15</f>
@@ -1323,67 +1319,43 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t>Despliegue / adopción
-(despliegue FFVV stock, Universidad Vida)</t>
-        </is>
-      </c>
-      <c r="B16" s="21" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="C16" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="D16" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="E16" s="21" t="n">
-        <v>12</v>
-      </c>
-      <c r="F16" s="21" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="G16" s="22">
-        <f>C16*$F$4</f>
-        <v/>
-      </c>
-      <c r="H16" s="22">
-        <f>D16*$F$4</f>
-        <v/>
-      </c>
-      <c r="I16" s="22">
-        <f>E16*$F$4</f>
-        <v/>
-      </c>
-      <c r="J16" s="21" t="n">
-        <v>2</v>
-      </c>
-      <c r="K16" s="21" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="L16" s="21">
-        <f>C16+$J16</f>
-        <v/>
-      </c>
-      <c r="M16" s="21">
-        <f>D16+$J16</f>
-        <v/>
-      </c>
-      <c r="N16" s="21">
-        <f>E16+$J16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
+          <t>🤝 Consultoría a otros equipos
+(agente AI App, Home) — se gestiona como SOPORTE, no como proyecto tallado</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="n"/>
+      <c r="K16" s="2" t="n"/>
+      <c r="L16" s="2" t="n"/>
+      <c r="M16" s="2" t="n"/>
+      <c r="N16" s="3" t="n"/>
+      <c r="O16" s="21" t="inlineStr">
+        <is>
+          <t>0.5–1h</t>
+        </is>
+      </c>
+      <c r="P16" s="21" t="inlineStr">
+        <is>
+          <t>2–4h</t>
+        </is>
+      </c>
+      <c r="Q16" s="21" t="inlineStr">
+        <is>
+          <t>1–2d</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
       <c r="A17" s="20" t="inlineStr">
         <is>
-          <t>Consultoría a otros equipos
-(agente AI App, Home) — se gestiona como SOPORTE, no como proyecto tallado</t>
+          <t>Soporte (desbloqueos, nuevos escenarios, QA conductual, deuda conductual)</t>
         </is>
       </c>
       <c r="B17" s="2" t="n"/>
@@ -1401,86 +1373,51 @@
       <c r="N17" s="3" t="n"/>
       <c r="O17" s="21" t="inlineStr">
         <is>
-          <t>0.5–1h</t>
-        </is>
-      </c>
-      <c r="P17" s="21" t="inlineStr">
-        <is>
-          <t>2–4h</t>
-        </is>
-      </c>
-      <c r="Q17" s="21" t="inlineStr">
-        <is>
-          <t>1–2d</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="20" t="inlineStr">
-        <is>
-          <t>Soporte (desbloqueos, nuevos escenarios, QA conductual, deuda conductual)</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n"/>
-      <c r="C18" s="2" t="n"/>
-      <c r="D18" s="2" t="n"/>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
-      <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="n"/>
-      <c r="J18" s="2" t="n"/>
-      <c r="K18" s="2" t="n"/>
-      <c r="L18" s="2" t="n"/>
-      <c r="M18" s="2" t="n"/>
-      <c r="N18" s="3" t="n"/>
-      <c r="O18" s="21" t="inlineStr">
-        <is>
           <t>Ver hoja «ANS Soporte»</t>
         </is>
       </c>
-      <c r="P18" s="2" t="n"/>
-      <c r="Q18" s="3" t="n"/>
-    </row>
-    <row r="20" ht="45" customHeight="1">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>📌 NOTAS: no hay fila de «DÍAS TOTALES por talla» — a diferencia del pipeline de Service Design, un quest de Behavioral Design normalmente es UN tipo de entregable, no la suma secuencial de todos. Si un quest combina 2 tipos (p.ej. research + modelo), suma solo esas dos filas. El appetite se recalibra cada trimestre con beholder_tools.py retro, no por negociación en el kickoff.</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
-      <c r="J20" s="2" t="n"/>
-      <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="n"/>
-      <c r="M20" s="2" t="n"/>
-      <c r="N20" s="2" t="n"/>
-      <c r="O20" s="2" t="n"/>
-      <c r="P20" s="2" t="n"/>
-      <c r="Q20" s="3" t="n"/>
+      <c r="P17" s="2" t="n"/>
+      <c r="Q17" s="3" t="n"/>
+    </row>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>📌 NOTAS: las categorías son cajones por FUNCIÓN (qué trabajo hace el entregable), no por artefacto — lo nuevo del futuro cae en un cajón existente sin rediseñar la tabla. No hay fila de «DÍAS TOTALES por talla»: un quest de BD normalmente es UNA función, no la suma secuencial de todas. Si un quest combina 2 funciones (p.ej. research + framework), talla cada una por separado y suma solo esas dos filas. El appetite se recalibra cada trimestre con beholder_tools.py retro, no por negociación en el kickoff.</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="n"/>
+      <c r="J19" s="2" t="n"/>
+      <c r="K19" s="2" t="n"/>
+      <c r="L19" s="2" t="n"/>
+      <c r="M19" s="2" t="n"/>
+      <c r="N19" s="2" t="n"/>
+      <c r="O19" s="2" t="n"/>
+      <c r="P19" s="2" t="n"/>
+      <c r="Q19" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="16">
     <mergeCell ref="A17:N17"/>
-    <mergeCell ref="A18:N18"/>
     <mergeCell ref="A7:A9"/>
     <mergeCell ref="G4:Q4"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="F7:I7"/>
-    <mergeCell ref="O18:Q18"/>
     <mergeCell ref="J7:J9"/>
-    <mergeCell ref="A20:Q20"/>
+    <mergeCell ref="A16:N16"/>
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="B7:E7"/>
     <mergeCell ref="O7:Q7"/>
     <mergeCell ref="K7:N7"/>
+    <mergeCell ref="O17:Q17"/>
     <mergeCell ref="D5:Q5"/>
+    <mergeCell ref="A19:Q19"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A1:Q1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Aclarar las definiciones de talla S/M/L/XL en el Excel del ANS BD
Los rótulos comprimidos ("Reuso de plantilla/patrón", etc.) se
reemplazan por frases autoexplicativas: S = ajustar algo existente,
M = crear algo nuevo acotado, L = alcance amplio o con gate externo,
XL = programa completo E2E multicanal.
</commit_message>
<xml_diff>
--- a/reportes/ANS_Behavioral_Design_propuesta.xlsx
+++ b/reportes/ANS_Behavioral_Design_propuesta.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,6 +60,10 @@
       <b val="1"/>
       <color rgb="FF7030A0"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="FF000000"/>
+      <sz val="8"/>
     </font>
     <font>
       <color rgb="FF375623"/>
@@ -268,25 +272,25 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -907,26 +911,26 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="55" customHeight="1">
       <c r="A9" s="15" t="n"/>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>Reuso de plantilla/patrón</t>
+          <t>Ajustar algo que ya existe (se reusa una plantilla o patrón del equipo)</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>Producto o bloque nuevo</t>
+          <t>Crear algo nuevo, pero acotado: 1 producto, 1 canal o 1 bloque</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>Familia/canal completo</t>
+          <t>Alcance amplio: varios productos/touchpoints, o pasa por gate externo (legal/médico)</t>
         </is>
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>Programa/ecosistema E2E</t>
+          <t>Programa completo de punta a punta, multicanal (p. ej. ecosistema de entendimiento)</t>
         </is>
       </c>
       <c r="F9" s="17" t="inlineStr">

</xml_diff>

<commit_message>
Ajustar ANS BD con revisión experta y sumar hoja de ejemplos de tallaje
- El feedback+VB ahora escala por talla (S/M/L/XL) en vez de sumar el
  valor de la talla L a las cuatro por igual, que subestimaba el gate
  externo en L/XL y lo sobreestimaba en S/M.
- El factor de conversión monedas/día pasa de 0.67 (supuesto inicial) a
  0.72 (ratio ya calibrado con la retro del tablero), mismo principio de
  reference-class forecasting que sostiene el resto de la propuesta.
- Nueva hoja "Ejemplos de Tallaje" (2da pestaña): un ejemplo concreto por
  talla y categoría, anclado a quests reales del TABLERO_BEHOLDER.md
  (Q-6, Q-8, Q-9, Q-10, Q-14, Q-15, Q-16, Q-21, Q-23/24, Q-26/27, Q-30,
  Q-38, Q-39) y a fuentes del ledger de cronista donde aplica.
</commit_message>
<xml_diff>
--- a/reportes/ANS_Behavioral_Design_propuesta.xlsx
+++ b/reportes/ANS_Behavioral_Design_propuesta.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="ANS Behavioral Design" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ANS Soporte BD" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Ejemplos de Tallaje" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ANS Soporte BD" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -80,6 +81,11 @@
     <font>
       <color rgb="FF000000"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="10">
@@ -233,7 +239,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -292,6 +298,9 @@
     </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -658,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:T19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -670,14 +679,17 @@
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
     <col width="9" customWidth="1" min="12" max="12"/>
     <col width="9" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="9" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -701,12 +713,15 @@
       <c r="N1" s="2" t="n"/>
       <c r="O1" s="2" t="n"/>
       <c r="P1" s="2" t="n"/>
-      <c r="Q1" s="3" t="n"/>
+      <c r="Q1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
+      <c r="S1" s="2" t="n"/>
+      <c r="T1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Tallaje por TIPO DE ENTREGABLE (no por etapa de un pipeline fijo). Los días son un appetite —presupuesto que el equipo decide invertir y calibra con su propio historial (retro trimestral)— no un estimado derivado de descomponer tareas. Ver reportes/ans_behavioral_design.md para el respaldo (/trinidad) y el detalle completo.</t>
+          <t>Tallaje por TIPO DE ENTREGABLE (no por etapa de un pipeline fijo). Los días son un appetite —presupuesto que el equipo decide invertir y calibra con su propio historial (retro trimestral)— no un estimado derivado de descomponer tareas. Ver reportes/ans_behavioral_design.md para el respaldo (/trinidad) y el detalle completo; ejemplos concretos por talla en la hoja «Ejemplos de Tallaje».</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -724,7 +739,10 @@
       <c r="N2" s="2" t="n"/>
       <c r="O2" s="2" t="n"/>
       <c r="P2" s="2" t="n"/>
-      <c r="Q2" s="3" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -741,12 +759,12 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>0.67</t>
+          <t>0.72</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>← 1 🪙 ≈ 1.5 días efectivos (recalibrar cada trimestre con beholder_tools.py retro)</t>
+          <t>← ratio medio REAL calibrado con la retro del tablero (no el 0.67 supuesto inicial de 1🪙≈1.5d) — reference-class forecasting (F-31); recalibrar cada trimestre con beholder_tools.py retro</t>
         </is>
       </c>
       <c r="H4" s="2" t="n"/>
@@ -758,7 +776,10 @@
       <c r="N4" s="2" t="n"/>
       <c r="O4" s="2" t="n"/>
       <c r="P4" s="2" t="n"/>
-      <c r="Q4" s="3" t="n"/>
+      <c r="Q4" s="2" t="n"/>
+      <c r="R4" s="2" t="n"/>
+      <c r="S4" s="2" t="n"/>
+      <c r="T4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -785,7 +806,40 @@
       <c r="N5" s="2" t="n"/>
       <c r="O5" s="2" t="n"/>
       <c r="P5" s="2" t="n"/>
-      <c r="Q5" s="3" t="n"/>
+      <c r="Q5" s="2" t="n"/>
+      <c r="R5" s="2" t="n"/>
+      <c r="S5" s="2" t="n"/>
+      <c r="T5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>🔧 Ajuste v2 (revisión experta)</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="3" t="n"/>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>El feedback+VB ahora tiene columna propia por talla (antes se sumaba el valor de la talla L a las 4 tallas por igual): el driver «validación requerida» (§3.2) es justamente lo que hace crecer esa cifra en S→XL, así que debe escalar, no ser plano.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="n"/>
+      <c r="L6" s="2" t="n"/>
+      <c r="M6" s="2" t="n"/>
+      <c r="N6" s="2" t="n"/>
+      <c r="O6" s="2" t="n"/>
+      <c r="P6" s="2" t="n"/>
+      <c r="Q6" s="2" t="n"/>
+      <c r="R6" s="2" t="n"/>
+      <c r="S6" s="2" t="n"/>
+      <c r="T6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -811,26 +865,28 @@
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>Feedback + VB
-(días extra si hay gate externo)</t>
-        </is>
-      </c>
-      <c r="K7" s="12" t="inlineStr">
+          <t>Feedback + VB (días extra por talla)</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="n"/>
+      <c r="M7" s="3" t="n"/>
+      <c r="N7" s="12" t="inlineStr">
         <is>
           <t>Appetite total con feedback (días)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="n"/>
-      <c r="N7" s="3" t="n"/>
-      <c r="O7" s="13" t="inlineStr">
+      <c r="O7" s="2" t="n"/>
+      <c r="P7" s="2" t="n"/>
+      <c r="Q7" s="3" t="n"/>
+      <c r="R7" s="13" t="inlineStr">
         <is>
           <t>Referencia rápida
 (no requiere quest, va como soporte)</t>
         </is>
       </c>
-      <c r="P7" s="2" t="n"/>
-      <c r="Q7" s="3" t="n"/>
+      <c r="S7" s="2" t="n"/>
+      <c r="T7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n"/>
@@ -874,38 +930,57 @@
           <t>XL</t>
         </is>
       </c>
-      <c r="J8" s="14" t="n"/>
-      <c r="K8" s="12" t="inlineStr">
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="L8" s="12" t="inlineStr">
+      <c r="K8" s="6" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="M8" s="12" t="inlineStr">
+      <c r="L8" s="6" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
+      <c r="M8" s="6" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
       <c r="N8" s="12" t="inlineStr">
         <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="O8" s="12" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="P8" s="12" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="Q8" s="12" t="inlineStr">
+        <is>
           <t>XL</t>
         </is>
       </c>
-      <c r="O8" s="13" t="inlineStr">
+      <c r="R8" s="13" t="inlineStr">
         <is>
           <t>Sesión</t>
         </is>
       </c>
-      <c r="P8" s="13" t="inlineStr">
+      <c r="S8" s="13" t="inlineStr">
         <is>
           <t>Revisión</t>
         </is>
       </c>
-      <c r="Q8" s="13" t="inlineStr">
+      <c r="T8" s="13" t="inlineStr">
         <is>
           <t>Co-diseño</t>
         </is>
@@ -935,56 +1010,75 @@
       </c>
       <c r="F9" s="17" t="inlineStr">
         <is>
-          <t>días × 0.67</t>
+          <t>días × 0.72</t>
         </is>
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>días × 0.67</t>
+          <t>días × 0.72</t>
         </is>
       </c>
       <c r="H9" s="17" t="inlineStr">
         <is>
-          <t>días × 0.67</t>
+          <t>días × 0.72</t>
         </is>
       </c>
       <c r="I9" s="17" t="inlineStr">
         <is>
-          <t>días × 0.67</t>
-        </is>
-      </c>
-      <c r="J9" s="15" t="n"/>
-      <c r="K9" s="18" t="inlineStr">
+          <t>días × 0.72</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>0–1d: sin gate, o 1 revisor rápido (&lt;48h)</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>1–2d: feedback estándar de 1 stakeholder</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>2d: 1 gate externo (comité o revisión formal)</t>
+        </is>
+      </c>
+      <c r="M9" s="16" t="inlineStr">
+        <is>
+          <t>3d+: 2+ gates (legal, médico, comité)</t>
+        </is>
+      </c>
+      <c r="N9" s="18" t="inlineStr">
         <is>
           <t>ANS Base + Feedback</t>
         </is>
       </c>
-      <c r="L9" s="18" t="inlineStr">
+      <c r="O9" s="18" t="inlineStr">
         <is>
           <t>ANS Base + Feedback</t>
         </is>
       </c>
-      <c r="M9" s="18" t="inlineStr">
+      <c r="P9" s="18" t="inlineStr">
         <is>
           <t>ANS Base + Feedback</t>
         </is>
       </c>
-      <c r="N9" s="18" t="inlineStr">
+      <c r="Q9" s="18" t="inlineStr">
         <is>
           <t>ANS Base + Feedback</t>
         </is>
       </c>
-      <c r="O9" s="19" t="inlineStr">
+      <c r="R9" s="19" t="inlineStr">
         <is>
           <t>0.5–1h</t>
         </is>
       </c>
-      <c r="P9" s="19" t="inlineStr">
+      <c r="S9" s="19" t="inlineStr">
         <is>
           <t>2–4h</t>
         </is>
       </c>
-      <c r="Q9" s="19" t="inlineStr">
+      <c r="T9" s="19" t="inlineStr">
         <is>
           <t>1–2d</t>
         </is>
@@ -1026,22 +1120,31 @@
         <v/>
       </c>
       <c r="J10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K10" s="21">
-        <f>B10+$J10</f>
-        <v/>
-      </c>
-      <c r="L10" s="21">
-        <f>C10+$J10</f>
-        <v/>
-      </c>
-      <c r="M10" s="21">
-        <f>D10+$J10</f>
-        <v/>
+      <c r="M10" s="21" t="n">
+        <v>3</v>
       </c>
       <c r="N10" s="21">
-        <f>E10+$J10</f>
+        <f>B10+J10</f>
+        <v/>
+      </c>
+      <c r="O10" s="21">
+        <f>C10+K10</f>
+        <v/>
+      </c>
+      <c r="P10" s="21">
+        <f>D10+L10</f>
+        <v/>
+      </c>
+      <c r="Q10" s="21">
+        <f>E10+M10</f>
         <v/>
       </c>
     </row>
@@ -1081,22 +1184,31 @@
         <v/>
       </c>
       <c r="J11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K11" s="21">
-        <f>B11+$J11</f>
-        <v/>
-      </c>
-      <c r="L11" s="21">
-        <f>C11+$J11</f>
-        <v/>
-      </c>
-      <c r="M11" s="21">
-        <f>D11+$J11</f>
-        <v/>
+      <c r="M11" s="21" t="n">
+        <v>3</v>
       </c>
       <c r="N11" s="21">
-        <f>E11+$J11</f>
+        <f>B11+J11</f>
+        <v/>
+      </c>
+      <c r="O11" s="21">
+        <f>C11+K11</f>
+        <v/>
+      </c>
+      <c r="P11" s="21">
+        <f>D11+L11</f>
+        <v/>
+      </c>
+      <c r="Q11" s="21">
+        <f>E11+M11</f>
         <v/>
       </c>
     </row>
@@ -1136,22 +1248,31 @@
         <v/>
       </c>
       <c r="J12" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K12" s="21">
-        <f>B12+$J12</f>
-        <v/>
-      </c>
-      <c r="L12" s="21">
-        <f>C12+$J12</f>
-        <v/>
-      </c>
-      <c r="M12" s="21">
-        <f>D12+$J12</f>
-        <v/>
+      <c r="M12" s="21" t="n">
+        <v>3</v>
       </c>
       <c r="N12" s="21">
-        <f>E12+$J12</f>
+        <f>B12+J12</f>
+        <v/>
+      </c>
+      <c r="O12" s="21">
+        <f>C12+K12</f>
+        <v/>
+      </c>
+      <c r="P12" s="21">
+        <f>D12+L12</f>
+        <v/>
+      </c>
+      <c r="Q12" s="21">
+        <f>E12+M12</f>
         <v/>
       </c>
     </row>
@@ -1191,22 +1312,31 @@
         <v/>
       </c>
       <c r="J13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K13" s="21">
-        <f>B13+$J13</f>
-        <v/>
-      </c>
-      <c r="L13" s="21">
-        <f>C13+$J13</f>
-        <v/>
-      </c>
-      <c r="M13" s="21">
-        <f>D13+$J13</f>
-        <v/>
+      <c r="L13" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="M13" s="21" t="n">
+        <v>3</v>
       </c>
       <c r="N13" s="21">
-        <f>E13+$J13</f>
+        <f>B13+J13</f>
+        <v/>
+      </c>
+      <c r="O13" s="21">
+        <f>C13+K13</f>
+        <v/>
+      </c>
+      <c r="P13" s="21">
+        <f>D13+L13</f>
+        <v/>
+      </c>
+      <c r="Q13" s="21">
+        <f>E13+M13</f>
         <v/>
       </c>
     </row>
@@ -1246,22 +1376,31 @@
         <v/>
       </c>
       <c r="J14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K14" s="21">
-        <f>B14+$J14</f>
-        <v/>
-      </c>
-      <c r="L14" s="21">
-        <f>C14+$J14</f>
-        <v/>
-      </c>
-      <c r="M14" s="21">
-        <f>D14+$J14</f>
-        <v/>
+      <c r="M14" s="21" t="n">
+        <v>3</v>
       </c>
       <c r="N14" s="21">
-        <f>E14+$J14</f>
+        <f>B14+J14</f>
+        <v/>
+      </c>
+      <c r="O14" s="21">
+        <f>C14+K14</f>
+        <v/>
+      </c>
+      <c r="P14" s="21">
+        <f>D14+L14</f>
+        <v/>
+      </c>
+      <c r="Q14" s="21">
+        <f>E14+M14</f>
         <v/>
       </c>
     </row>
@@ -1301,22 +1440,31 @@
         <v/>
       </c>
       <c r="J15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K15" s="21">
-        <f>B15+$J15</f>
-        <v/>
-      </c>
-      <c r="L15" s="21">
-        <f>C15+$J15</f>
-        <v/>
-      </c>
-      <c r="M15" s="21">
-        <f>D15+$J15</f>
-        <v/>
+      <c r="M15" s="21" t="n">
+        <v>3</v>
       </c>
       <c r="N15" s="21">
-        <f>E15+$J15</f>
+        <f>B15+J15</f>
+        <v/>
+      </c>
+      <c r="O15" s="21">
+        <f>C15+K15</f>
+        <v/>
+      </c>
+      <c r="P15" s="21">
+        <f>D15+L15</f>
+        <v/>
+      </c>
+      <c r="Q15" s="21">
+        <f>E15+M15</f>
         <v/>
       </c>
     </row>
@@ -1339,18 +1487,21 @@
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="n"/>
       <c r="M16" s="2" t="n"/>
-      <c r="N16" s="3" t="n"/>
-      <c r="O16" s="21" t="inlineStr">
+      <c r="N16" s="2" t="n"/>
+      <c r="O16" s="2" t="n"/>
+      <c r="P16" s="2" t="n"/>
+      <c r="Q16" s="3" t="n"/>
+      <c r="R16" s="21" t="inlineStr">
         <is>
           <t>0.5–1h</t>
         </is>
       </c>
-      <c r="P16" s="21" t="inlineStr">
+      <c r="S16" s="21" t="inlineStr">
         <is>
           <t>2–4h</t>
         </is>
       </c>
-      <c r="Q16" s="21" t="inlineStr">
+      <c r="T16" s="21" t="inlineStr">
         <is>
           <t>1–2d</t>
         </is>
@@ -1374,14 +1525,17 @@
       <c r="K17" s="2" t="n"/>
       <c r="L17" s="2" t="n"/>
       <c r="M17" s="2" t="n"/>
-      <c r="N17" s="3" t="n"/>
-      <c r="O17" s="21" t="inlineStr">
-        <is>
-          <t>Ver hoja «ANS Soporte»</t>
-        </is>
-      </c>
+      <c r="N17" s="2" t="n"/>
+      <c r="O17" s="2" t="n"/>
       <c r="P17" s="2" t="n"/>
       <c r="Q17" s="3" t="n"/>
+      <c r="R17" s="21" t="inlineStr">
+        <is>
+          <t>Ver hoja «ANS Soporte»</t>
+        </is>
+      </c>
+      <c r="S17" s="2" t="n"/>
+      <c r="T17" s="3" t="n"/>
     </row>
     <row r="19" ht="45" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
@@ -1404,32 +1558,314 @@
       <c r="N19" s="2" t="n"/>
       <c r="O19" s="2" t="n"/>
       <c r="P19" s="2" t="n"/>
-      <c r="Q19" s="3" t="n"/>
+      <c r="Q19" s="2" t="n"/>
+      <c r="R19" s="2" t="n"/>
+      <c r="S19" s="2" t="n"/>
+      <c r="T19" s="3" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
-    <mergeCell ref="A17:N17"/>
+  <mergeCells count="18">
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="A17:Q17"/>
     <mergeCell ref="A7:A9"/>
-    <mergeCell ref="G4:Q4"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="F7:I7"/>
-    <mergeCell ref="J7:J9"/>
-    <mergeCell ref="A16:N16"/>
-    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="G4:T4"/>
+    <mergeCell ref="R7:T7"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="D6:T6"/>
+    <mergeCell ref="R17:T17"/>
+    <mergeCell ref="N7:Q7"/>
     <mergeCell ref="B7:E7"/>
-    <mergeCell ref="O7:Q7"/>
-    <mergeCell ref="K7:N7"/>
-    <mergeCell ref="O17:Q17"/>
-    <mergeCell ref="D5:Q5"/>
-    <mergeCell ref="A19:Q19"/>
+    <mergeCell ref="A16:Q16"/>
+    <mergeCell ref="A2:T2"/>
     <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="D5:T5"/>
+    <mergeCell ref="A19:T19"/>
+    <mergeCell ref="J7:M7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ejemplos de Tallaje — Behavioral Design (por categoría funcional)</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="3" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Un ejemplo concreto por talla y categoría, para calibrar el juicio antes de tallar un quest nuevo (driver 3.2: novedad · superficie · validación requerida). Mezcla trabajo YA ENTREGADO —con su clave del tablero (Q-n) para trazabilidad— y trabajo FUTURO (marcado «futuro»), porque las categorías son cajones por función, no por artefacto hecho hasta hoy. Días y monedas exactos están en la hoja anterior; aquí solo el criterio cualitativo. Fuentes citadas: ver research/fuentes/registro_fuentes.md (ID F-n).</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Categoría (función)</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Ejemplo concreto por talla</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="n"/>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="110" customHeight="1">
+      <c r="A6" s="23" t="inlineStr">
+        <is>
+          <t>🔍 Evidencia y diagnóstico</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Desk research acotado sobre un tema puntual para informar una decisión rápida — p. ej. bench de 3–4 aseguradoras sobre cómo comunican el copago EPS, antes de definir el ángulo de una guía (futuro).</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Bench + síntesis con hipótesis — Q-6: desk research + bench de estrategias de contacto en frío vs. caliente para la mesa Back to Basics (qué gatillos abren conversación: reciprocidad, curiosidad, personalización).</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Research con entrevistas u observación — análogo a Q-21 (Evolution+ Cobranzas): mapear barreras y motivaciones de un perfil de pagador B2B con entrevistas a analistas de cuentas por cobrar, no solo desk research.</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Diagnóstico E2E con data + campo — levantar el diagnóstico de barreras de entendimiento del journey EPS completo (multiempresa + individual), cruzando NPS/CSAT con entrevistas, como insumo del Ecosistema EPS (Q-38) (futuro).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="110" customHeight="1">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>📣 Comunicación conductual</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Ajuste de copy sobre una plantilla que ya existe — adaptar el copy de un WhatsApp de primer contacto ya validado a un nuevo segmento de asesores (futuro).</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Pieza o set nuevo para 1 canal con validación — Q-16: 6 guías resumidas AMI en PDF; simplificación radical de la póliza (lenguaje claro, jerarquía de coberturas) validada con Producto y equipo médico. Ataca la sobrecarga informativa, causa #1 de desconfianza (F-1, tenencia SBS 2023).</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Familia de piezas o journey multicanal con gate legal — Q-10: plantillas de WhatsApp y correo de primer contacto CON CUA, que pasan por el gate de Legal/Cumplimiento antes de salir (marco Ley 32323, F-28).</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Ecosistema de comunicación E2E — rediseñar guías + cartas + notificaciones del journey de renovación EPS como sistema coherente, no piezas sueltas (futuro).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="110" customHeight="1">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>🎛️ Arquitectura de intervención</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Micro-fricción o default en un paso existente — reordenar las opciones de un formulario de renovación para que el default sea la cobertura recomendada (futuro).</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Intervención en un momento de decisión puntual — rediseñar el paso de checkout de un producto EPS con framing de pérdida en vez de ganancia (futuro).</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Estrategia conductual de un flujo completo — Q-9: informe con la arquitectura de decisión del primer contacto (canal, momento, mensaje) validada por CUA, Cumplimiento y Legal; +20–30% agendamiento de citas (est.).</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Programa conductual E2E / arquitectura de un producto — Q-38: diseño To Be del Ecosistema de entendimiento y uso eficiente de seguros EPS, con touchpoints a lo largo de todo el journey del asegurado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="110" customHeight="1">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>🧪 Validación y experimentación</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Test guerrilla / sacrificial concepts — Q-8: 6 sacrificial concepts de contacto a no clientes sin CUA, para elicitar objeciones reales antes de invertir en el diseño final (preferencias reveladas, no declaradas).</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Test moderado con artefactos — Q-26/Q-27: plan de testeo + artefactos tangibles de Vivo Pack, con hipótesis de comprensión y disposición a pagar.</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Experimento A/B con tracking — Q-23/Q-24: diseño y ejecución de piloto de conciliación B2B; grupo tratamiento vs. control midiendo conducta real (conciliación a tiempo), no intención declarada.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Programa de experimentación en serie — batería trimestral de experimentos A/B sobre distintos momentos del journey de renovación, con backlog priorizado y aprendizaje acumulado entre rondas (futuro). Ojo: un solo piloto de wellness no prueba impacto en siniestralidad (F-26) — el programa necesita varias rondas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="110" customHeight="1">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>📚 Sistemas y frameworks</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Ajuste de una sección de un playbook existente — actualizar el capítulo de objeciones del playbook de ventas con hallazgos de un research reciente (futuro).</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Bloque nuevo o framework adaptado — Q-30: playbook del servicio Bienestar 360, codificando el modelo de cambio de hábitos del programa para hacerlo replicable.</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Playbook o modelo completo con validación — Q-5: modelo de competencias de Universidad Vida (niveles, calendarización con práctica espaciada F-16, evaluación con reconocimiento F-18), validado con Learning.</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Sistema con evaluación y gobernanza — Q-39: modelo de entendimiento y uso eficiente de seguros del Chapter, con métricas propias y gobierno de actualización entre proyectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="110" customHeight="1">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>🚀 Adopción y despliegue</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Sesión de capacitación con material ya listo — kickoff con un equipo comercial explicando una guía resumida ya publicada (futuro).</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>1 cohorte con materiales listos — Q-14: despliegue del playbook de storytelling con la cohorte de asesores de FFVV stock.</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Multi-cohorte con campeones y refuerzos — Q-15: despliegue de Universidad Vida por cohortes sucesivas, con hitos visibles y refuerzo social para sostener el hábito formativo más allá del lanzamiento (F-18, reconocimiento + feedback).</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Organización completa con medición de adopción — campaña de adopción del Ecosistema EPS a nivel de toda la fuerza comercial (multiempresa + individual), con tracking de uso post-lanzamiento en NPS/CSAT (futuro, ligado a Q-38).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>🤝 Consultoría a otros equipos</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Se gestiona como soporte por horas (ver hoja «ANS Soporte BD»): sesión puntual, revisión de un artefacto ajeno, o co-diseño acotado con el agente AI de App/Home. No se talla como quest propio — si crece más allá de eso, se abre un quest en la categoría que corresponda por función.</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="3" t="n"/>
+    </row>
+    <row r="14" ht="55" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>📌 Cómo leer esta hoja: los ejemplos «futuro» son hipotéticos —trabajo que cabe en la categoría aunque el equipo no lo haya hecho todavía— y sirven para probar que el cajón por función no se rompe con lo nuevo. Los marcados con Q-n ya ocurrieron y están en TABLERO_BEHOLDER.md; úsalos como ancla de calibración en la retro trimestral (reference-class forecasting, F-31) en vez de discutir la talla desde cero cada vez.</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A14:E14"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Sincronizar hoja Ejemplos de Tallaje con Q-48 y el caso de alineación EPS
- El ejemplo L de Evidencia y diagnóstico ahora cita Q-48 (modelo de
  retención con Edu Rebata, Alejandro) en vez del hipotético genérico
  que tenía antes — ya es un quest real del tablero.
- Sistemas y frameworks (L) y Consultoría suman el caso de dar inputs
  conductuales a los equipos dueños del Ecosistema EPS (CX, mkt, guías,
  App), como ejemplo de la regla de encaje: el framework se talla en
  Sistemas, la alineación con los 4 equipos se talla aparte en soporte.
</commit_message>
<xml_diff>
--- a/reportes/ANS_Behavioral_Design_propuesta.xlsx
+++ b/reportes/ANS_Behavioral_Design_propuesta.xlsx
@@ -1664,7 +1664,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="110" customHeight="1">
+    <row r="6" ht="125" customHeight="1">
       <c r="A6" s="23" t="inlineStr">
         <is>
           <t>🔍 Evidencia y diagnóstico</t>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Research con entrevistas u observación — análogo a Q-21 (Evolution+ Cobranzas): mapear barreras y motivaciones de un perfil de pagador B2B con entrevistas a analistas de cuentas por cobrar, no solo desk research.</t>
+          <t>Research con entrevistas u observación — Q-21 (Evolution+ Cobranzas): mapear barreras y motivaciones de un perfil de pagador B2B con entrevistas a analistas de cuentas por cobrar, no solo desk research. Mismo tier: Q-48, cruzar data de renovación + siniestros para el modelo de retención en salud con Edu Rebata (Alejandro) — el riesgo es el acceso cross-área, no el análisis (se mide como Lead time, no Reloj BD).</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
@@ -1691,7 +1691,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="110" customHeight="1">
+    <row r="7" ht="125" customHeight="1">
       <c r="A7" s="23" t="inlineStr">
         <is>
           <t>📣 Comunicación conductual</t>
@@ -1718,7 +1718,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="110" customHeight="1">
+    <row r="8" ht="125" customHeight="1">
       <c r="A8" s="23" t="inlineStr">
         <is>
           <t>🎛️ Arquitectura de intervención</t>
@@ -1745,7 +1745,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="110" customHeight="1">
+    <row r="9" ht="125" customHeight="1">
       <c r="A9" s="23" t="inlineStr">
         <is>
           <t>🧪 Validación y experimentación</t>
@@ -1772,7 +1772,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="110" customHeight="1">
+    <row r="10" ht="125" customHeight="1">
       <c r="A10" s="23" t="inlineStr">
         <is>
           <t>📚 Sistemas y frameworks</t>
@@ -1795,11 +1795,11 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Sistema con evaluación y gobernanza — Q-39: modelo de entendimiento y uso eficiente de seguros del Chapter, con métricas propias y gobierno de actualización entre proyectos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="110" customHeight="1">
+          <t>Sistema con evaluación y gobernanza — Q-39: modelo de entendimiento y uso eficiente de seguros del Chapter, con métricas propias y gobierno de actualización entre proyectos. Mismo tier: inputs conductuales para que CX (journey), mkt (pauta), guías y App construyan sus propias piezas del Ecosistema EPS (futuro, ligado a Q-38) — el framework se talla aquí; alinear a los 4 equipos dueños se talla aparte en 🤝 Consultoría (regla de encaje).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="125" customHeight="1">
       <c r="A11" s="23" t="inlineStr">
         <is>
           <t>🚀 Adopción y despliegue</t>
@@ -1834,7 +1834,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Se gestiona como soporte por horas (ver hoja «ANS Soporte BD»): sesión puntual, revisión de un artefacto ajeno, o co-diseño acotado con el agente AI de App/Home. No se talla como quest propio — si crece más allá de eso, se abre un quest en la categoría que corresponda por función.</t>
+          <t>Se gestiona como soporte por horas (ver hoja «ANS Soporte BD»): sesión puntual, revisión de un artefacto ajeno, o co-diseño acotado con el agente AI de App/Home. No se talla como quest propio — si crece más allá de eso, se abre un quest en la categoría que corresponda por función. Caso real de escala: alinear a 4 equipos dueños (CX, mkt, guías, App) del Ecosistema EPS son 4 revisiones de 2–4h, no 1 — avisar si esto se come la bolsa mensual de ~8h/persona (§3.3).</t>
         </is>
       </c>
       <c r="C12" s="2" t="n"/>

</xml_diff>

<commit_message>
Aclarar que el Acompañamiento embebido tiene dos fases, no una bolsa de 6 meses
El ANS de capacidad reservada de §3.7 aplica solo mientras dura la
exploración. En cuanto el proyecto prioriza sus soluciones en un
roadmap, las que le corresponden a BD dejan de ser "capacidad
reservada" y vuelven al catálogo normal de entregables (3.1) — se
tallan, tienen sus propios drivers (3.2) y su propio par de relojes
(3.4), igual que cualquier quest que hubiera entrado por la puerta de
un entregable puntual.

- ans_behavioral_design.md: reestructura 3.7 en dos fases explícitas
  (exploración vs. roadmap) y ajusta el punto 6 del resumen ejecutivo.
- Excel: nota de la fila "Acompañamiento" ahora describe ambas fases;
  los ejemplos L/XL de "Ejemplos de Tallaje" muestran el momento exacto
  en que EPIC-1 y EPIC-7 hicieron esa transición en la práctica.
</commit_message>
<xml_diff>
--- a/reportes/ANS_Behavioral_Design_propuesta.xlsx
+++ b/reportes/ANS_Behavioral_Design_propuesta.xlsx
@@ -1521,11 +1521,11 @@
       <c r="S16" s="2" t="n"/>
       <c r="T16" s="3" t="n"/>
     </row>
-    <row r="17" ht="55" customHeight="1">
+    <row r="17" ht="68" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
           <t>🧭 Acompañamiento de proyecto (embebido E2E)
-(BD entra desde la exploración de un proyecto de negocio, acompaña definición de soluciones y diseño, y CIERRA delegando el diseño/fix a quien lo implementa — no lo despliega BD. Puede durar hasta 6 meses; se re-compromete cada trimestre, no una sola vez)</t>
+(FASE 1 — exploración: BD entra desde el inicio de un proyecto de negocio sin entregable definido todavía; ANS de capacidad reservada, tabla de la derecha. FASE 2 — roadmap: en cuanto el proyecto prioriza sus soluciones, las que corresponden a BD vuelven al catálogo normal ⬆️ y se tallan como cualquier entregable — el acompañamiento no dura los 6 meses completos, solo hasta que existe roadmap)</t>
         </is>
       </c>
       <c r="B17" s="21" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="R17" s="25" t="inlineStr">
         <is>
-          <t>Talla = % de capacidad reservada, no días de un entregable</t>
+          <t>Talla = % de capacidad reservada SOLO en fase de exploración (antes del roadmap)</t>
         </is>
       </c>
       <c r="S17" s="2" t="n"/>
@@ -1991,7 +1991,7 @@
       <c r="A13" s="26" t="inlineStr">
         <is>
           <t>🧭 Acompañamiento de proyecto
-(embebido E2E)</t>
+(embebido E2E, solo fase de exploración)</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -2006,12 +2006,12 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>L (5–6 🪙/trim.): hilo conductor a través de la mayoría de las funciones — EPIC-7 Renovación EPS: guías (📣) → validación → entrega → Diseño To Be del ecosistema (🎛️), ahora extendido por Q-48 (🔍) sin fecha de cierre.</t>
+          <t>L (5–6 🪙/trim.): hilo conductor a través de la mayoría de las funciones mientras no hay roadmap — p. ej. la fase inicial de EPIC-7 antes de Q-35 (entender qué necesitaba el negocio de EPS). En cuanto salió el roadmap, las guías (📣), la validación y el Diseño To Be (🎛️) se tallaron normal por 3.1 — ya no como acompañamiento.</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>XL (7–8 🪙/trim.): casi dedicación completa con pairing — EPIC-1 Mesa Back to Basics: research (🔍) → sacrificial concepts (🧪) → informe CUA (🎛️) → materiales (📣) → AIDA (📚) → despliegue FFVV (🚀); 10 semanas, 3 personas, 25 🪙 en total.</t>
+          <t>XL (7–8 🪙/trim.): casi dedicación completa con pairing, solo mientras dura la exploración — p. ej. las primeras semanas de EPIC-1 Mesa Back to Basics (research + validación + sacrificial concepts, Q-6/7/8) antes del informe CUA. En cuanto el informe priorizó soluciones, plantillas (📣), AIDA (📚) y despliegue (🚀) pasaron a tallarse como quests normales de 3.1 — el acompañamiento como tal ya había cerrado.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Quitar las claves Q-n del Excel de ANS Behavioral Design
Los ejemplos de la hoja "Ejemplos de Tallaje" citaban códigos internos
del tablero Beholder (Q-6, Q-9, Q-38, etc.) que no significan nada fuera
de ese tablero. El Excel del ANS es un documento para uso externo (con
Milagros y el comité), así que los ejemplos ahora describen el trabajo
por su nombre y contenido en vez de por su clave interna — el contenido
sustantivo de cada ejemplo no cambia, solo se desacopla de la
nomenclatura Q-n.
</commit_message>
<xml_diff>
--- a/reportes/ANS_Behavioral_Design_propuesta.xlsx
+++ b/reportes/ANS_Behavioral_Design_propuesta.xlsx
@@ -1768,7 +1768,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Un ejemplo concreto por talla y categoría, para calibrar el juicio antes de tallar un quest nuevo (driver 3.2: novedad · superficie · validación requerida). Mezcla trabajo YA ENTREGADO —con su clave del tablero (Q-n) para trazabilidad— y trabajo FUTURO (marcado «futuro»), porque las categorías son cajones por función, no por artefacto hecho hasta hoy. Días y monedas exactos están en la hoja anterior; aquí solo el criterio cualitativo. Fuentes citadas: ver research/fuentes/registro_fuentes.md (ID F-n).</t>
+          <t>Un ejemplo concreto por talla y categoría, para calibrar el juicio antes de tallar un quest nuevo (driver 3.2: novedad · superficie · validación requerida). Mezcla trabajo YA ENTREGADO (con su nombre, para trazabilidad) y trabajo FUTURO (marcado «futuro»), porque las categorías son cajones por función, no por artefacto hecho hasta hoy. Días y monedas exactos están en la hoja anterior; aquí solo el criterio cualitativo. Fuentes citadas: ver research/fuentes/registro_fuentes.md (ID F-n).</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1827,17 +1827,17 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Bench + síntesis con hipótesis — Q-6: desk research + bench de estrategias de contacto en frío vs. caliente para la mesa Back to Basics (qué gatillos abren conversación: reciprocidad, curiosidad, personalización).</t>
+          <t>Bench + síntesis con hipótesis — desk research + bench de estrategias de contacto en frío vs. caliente para la mesa Back to Basics (qué gatillos abren conversación: reciprocidad, curiosidad, personalización).</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Research con entrevistas u observación — Q-21 (Evolution+ Cobranzas): mapear barreras y motivaciones de un perfil de pagador B2B con entrevistas a analistas de cuentas por cobrar, no solo desk research. Mismo tier: Q-48, cruzar data de renovación + siniestros para el modelo de retención en salud con Edu Rebata (Alejandro) — el riesgo es el acceso cross-área, no el análisis (se mide como Lead time, no Reloj BD).</t>
+          <t>Research con entrevistas u observación — mapear barreras y motivaciones de un perfil de pagador B2B con entrevistas a analistas de cuentas por cobrar (Evolution+ Cobranzas), no solo desk research. Mismo tier: cruzar data de renovación + siniestros para el modelo de retención en salud con Edu Rebata (Alejandro) — el riesgo es el acceso cross-área, no el análisis (se mide como Lead time, no Reloj BD).</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Diagnóstico E2E con data + campo — levantar el diagnóstico de barreras de entendimiento del journey EPS completo (multiempresa + individual), cruzando NPS/CSAT con entrevistas, como insumo del Ecosistema EPS (Q-38) (futuro).</t>
+          <t>Diagnóstico E2E con data + campo — levantar el diagnóstico de barreras de entendimiento del journey EPS completo (multiempresa + individual), cruzando NPS/CSAT con entrevistas, como insumo del Ecosistema EPS (futuro).</t>
         </is>
       </c>
     </row>
@@ -1854,12 +1854,12 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Pieza o set nuevo para 1 canal con validación — Q-16: 6 guías resumidas AMI en PDF; simplificación radical de la póliza (lenguaje claro, jerarquía de coberturas) validada con Producto y equipo médico. Ataca la sobrecarga informativa, causa #1 de desconfianza (F-1, tenencia SBS 2023).</t>
+          <t>Pieza o set nuevo para 1 canal con validación — 6 guías resumidas AMI en PDF; simplificación radical de la póliza (lenguaje claro, jerarquía de coberturas) validada con Producto y equipo médico. Ataca la sobrecarga informativa, causa #1 de desconfianza (F-1, tenencia SBS 2023).</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Familia de piezas o journey multicanal con gate legal — Q-10: plantillas de WhatsApp y correo de primer contacto CON CUA, que pasan por el gate de Legal/Cumplimiento antes de salir (marco Ley 32323, F-28).</t>
+          <t>Familia de piezas o journey multicanal con gate legal — plantillas de WhatsApp y correo de primer contacto CON CUA, que pasan por el gate de Legal/Cumplimiento antes de salir (marco Ley 32323, F-28).</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -1886,12 +1886,12 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Estrategia conductual de un flujo completo — Q-9: informe con la arquitectura de decisión del primer contacto (canal, momento, mensaje) validada por CUA, Cumplimiento y Legal; +20–30% agendamiento de citas (est.).</t>
+          <t>Estrategia conductual de un flujo completo — informe con la arquitectura de decisión del primer contacto (canal, momento, mensaje) validada por CUA, Cumplimiento y Legal; +20–30% agendamiento de citas (est.).</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Programa conductual E2E / arquitectura de un producto — Q-38: diseño To Be del Ecosistema de entendimiento y uso eficiente de seguros EPS, con touchpoints a lo largo de todo el journey del asegurado.</t>
+          <t>Programa conductual E2E / arquitectura de un producto — diseño To Be del Ecosistema de entendimiento y uso eficiente de seguros EPS, con touchpoints a lo largo de todo el journey del asegurado.</t>
         </is>
       </c>
     </row>
@@ -1903,17 +1903,17 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Test guerrilla / sacrificial concepts — Q-8: 6 sacrificial concepts de contacto a no clientes sin CUA, para elicitar objeciones reales antes de invertir en el diseño final (preferencias reveladas, no declaradas).</t>
+          <t>Test guerrilla / sacrificial concepts — 6 sacrificial concepts de contacto a no clientes sin CUA, para elicitar objeciones reales antes de invertir en el diseño final (preferencias reveladas, no declaradas).</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Test moderado con artefactos — Q-26/Q-27: plan de testeo + artefactos tangibles de Vivo Pack, con hipótesis de comprensión y disposición a pagar.</t>
+          <t>Test moderado con artefactos — plan de testeo + artefactos tangibles de Vivo Pack, con hipótesis de comprensión y disposición a pagar.</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Experimento A/B con tracking — Q-23/Q-24: diseño y ejecución de piloto de conciliación B2B; grupo tratamiento vs. control midiendo conducta real (conciliación a tiempo), no intención declarada.</t>
+          <t>Experimento A/B con tracking — diseño y ejecución de piloto de conciliación B2B; grupo tratamiento vs. control midiendo conducta real (conciliación a tiempo), no intención declarada.</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -1935,17 +1935,17 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Bloque nuevo o framework adaptado — Q-30: playbook del servicio Bienestar 360, codificando el modelo de cambio de hábitos del programa para hacerlo replicable.</t>
+          <t>Bloque nuevo o framework adaptado — playbook del servicio Bienestar 360, codificando el modelo de cambio de hábitos del programa para hacerlo replicable.</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Playbook o modelo completo con validación — Q-5: modelo de competencias de Universidad Vida (niveles, calendarización con práctica espaciada F-16, evaluación con reconocimiento F-18), validado con Learning.</t>
+          <t>Playbook o modelo completo con validación — modelo de competencias de Universidad Vida (niveles, calendarización con práctica espaciada F-16, evaluación con reconocimiento F-18), validado con Learning.</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Sistema con evaluación y gobernanza — Q-39: modelo de entendimiento y uso eficiente de seguros del Chapter, con métricas propias y gobierno de actualización entre proyectos. Mismo tier: inputs conductuales para que CX (journey), mkt (pauta), guías y App construyan sus propias piezas del Ecosistema EPS (futuro, ligado a Q-38) — el framework se talla aquí; alinear a los 4 equipos dueños se talla aparte en 🤝 Consultoría (regla de encaje).</t>
+          <t>Sistema con evaluación y gobernanza — modelo de entendimiento y uso eficiente de seguros del Chapter, con métricas propias y gobierno de actualización entre proyectos. Mismo tier: inputs conductuales para que CX (journey), mkt (pauta), guías y App construyan sus propias piezas del Ecosistema EPS (futuro) — el framework se talla aquí; alinear a los 4 equipos dueños se talla aparte en 🤝 Consultoría (regla de encaje).</t>
         </is>
       </c>
     </row>
@@ -1962,17 +1962,17 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>1 cohorte con materiales listos — Q-14: despliegue del playbook de storytelling con la cohorte de asesores de FFVV stock.</t>
+          <t>1 cohorte con materiales listos — despliegue del playbook de storytelling con la cohorte de asesores de FFVV stock.</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Multi-cohorte con campeones y refuerzos — Q-15: despliegue de Universidad Vida por cohortes sucesivas, con hitos visibles y refuerzo social para sostener el hábito formativo más allá del lanzamiento (F-18, reconocimiento + feedback).</t>
+          <t>Multi-cohorte con campeones y refuerzos — despliegue de Universidad Vida por cohortes sucesivas, con hitos visibles y refuerzo social para sostener el hábito formativo más allá del lanzamiento (F-18, reconocimiento + feedback).</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Organización completa con medición de adopción — campaña de adopción del Ecosistema EPS a nivel de toda la fuerza comercial (multiempresa + individual), con tracking de uso post-lanzamiento en NPS/CSAT (futuro, ligado a Q-38).</t>
+          <t>Organización completa con medición de adopción — campaña de adopción del Ecosistema EPS a nivel de toda la fuerza comercial (multiempresa + individual), con tracking de uso post-lanzamiento en NPS/CSAT (futuro).</t>
         </is>
       </c>
     </row>
@@ -1996,22 +1996,22 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>S (1–2 🪙/trim.): check-ins puntuales con un proyecto que recién explora — p. ej. consultoría breve y recurrente con Convenios mientras entienden su modelo de venta actual (Q-32), sin research ni entregable propio de BD todavía (futuro).</t>
+          <t>S (1–2 🪙/trim.): check-ins puntuales con un proyecto que recién explora — p. ej. consultoría breve y recurrente con Convenios mientras entienden su modelo de venta actual, sin research ni entregable propio de BD todavía (futuro).</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>M (3–4 🪙/trim.): participación activa en 2–3 funciones — p. ej. acompañar Spark: Vivo Pack desde el research hasta el testeo de concepto (Q-26/27/28), sin llegar a diseño de intervención ni despliegue.</t>
+          <t>M (3–4 🪙/trim.): participación activa en 2–3 funciones — p. ej. acompañar Spark: Vivo Pack desde el research hasta el testeo de concepto, sin llegar a diseño de intervención ni despliegue.</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>L (5–6 🪙/trim.): hilo conductor a través de la mayoría de las funciones mientras no hay roadmap — p. ej. la fase inicial de EPIC-7 antes de Q-35 (entender qué necesitaba el negocio de EPS). En cuanto salió el roadmap, las guías (📣), la validación y el Diseño To Be (🎛️) se tallaron normal por 3.1 — ya no como acompañamiento.</t>
+          <t>L (5–6 🪙/trim.): hilo conductor a través de la mayoría de las funciones mientras no hay roadmap — p. ej. la fase inicial de la Renovación EPS (entender qué necesitaba el negocio de EPS, antes de que existieran las guías). En cuanto salió el roadmap, las guías (📣), la validación y el Diseño To Be (🎛️) se tallaron normal por 3.1 — ya no como acompañamiento.</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>XL (7–8 🪙/trim.): casi dedicación completa con pairing, solo mientras dura la exploración — p. ej. las primeras semanas de EPIC-1 Mesa Back to Basics (research + validación + sacrificial concepts, Q-6/7/8) antes del informe CUA. En cuanto el informe priorizó soluciones, plantillas (📣), AIDA (📚) y despliegue (🚀) pasaron a tallarse como quests normales de 3.1 — el acompañamiento como tal ya había cerrado.</t>
+          <t>XL (7–8 🪙/trim.): casi dedicación completa con pairing, solo mientras dura la exploración — p. ej. las primeras semanas de la Mesa Back to Basics (research + validación + sacrificial concepts de estrategias de contacto) antes del informe CUA. En cuanto el informe priorizó soluciones, plantillas (📣), AIDA (📚) y despliegue (🚀) pasaron a tallarse como quests normales de 3.1 — el acompañamiento como tal ya había cerrado.</t>
         </is>
       </c>
     </row>
@@ -2033,7 +2033,7 @@
     <row r="17" ht="55" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>📌 Cómo leer esta hoja: los ejemplos «futuro» son hipotéticos —trabajo que cabe en la categoría aunque el equipo no lo haya hecho todavía— y sirven para probar que el cajón por función no se rompe con lo nuevo. Los marcados con Q-n ya ocurrieron y están en TABLERO_BEHOLDER.md; úsalos como ancla de calibración en la retro trimestral (reference-class forecasting, F-31) en vez de discutir la talla desde cero cada vez.</t>
+          <t>📌 Cómo leer esta hoja: los ejemplos «futuro» son hipotéticos —trabajo que cabe en la categoría aunque el equipo no lo haya hecho todavía— y sirven para probar que el cajón por función no se rompe con lo nuevo. Los que no dicen «futuro» ya ocurrieron; úsalos como ancla de calibración en la retro trimestral (reference-class forecasting, F-31) en vez de discutir la talla desde cero cada vez.</t>
         </is>
       </c>
       <c r="B17" s="2" t="n"/>

</xml_diff>

<commit_message>
Reordenar la hoja principal del ANS por feedback de Melissa: monedas al final
Las monedas se calculaban del día BASE (columna a mitad de la fila),
así que el equivalente en monedas del appetite total (base + feedback)
había que sacarlo por fuera de la hoja. Melissa pidió un solo campo al
final con fórmula (total de días × factor del equipo).

Reordena la fila principal a base (días) → feedback (días) → total
(días) → monedas del total, todo encadenado con fórmula: J=B+F,
N=J*$F$4. Se lee de una sola pasada: construyo → valido → total en
días → total en monedas.
</commit_message>
<xml_diff>
--- a/reportes/ANS_Behavioral_Design_propuesta.xlsx
+++ b/reportes/ANS_Behavioral_Design_propuesta.xlsx
@@ -137,12 +137,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF4B942"/>
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor rgb="FFF4B942"/>
       </patternFill>
     </fill>
     <fill>
@@ -282,10 +282,10 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -296,10 +296,10 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -317,7 +317,7 @@
     <xf numFmtId="0" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -841,14 +841,14 @@
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>🔧 Ajuste v2 (revisión experta)</t>
+          <t>🔧 Ajuste v3 (feedback de Melissa)</t>
         </is>
       </c>
       <c r="B6" s="2" t="n"/>
       <c r="C6" s="3" t="n"/>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>El feedback+VB ahora tiene columna propia por talla (antes se sumaba el valor de la talla L a las 4 tallas por igual): el driver «validación requerida» (§3.2) es justamente lo que hace crecer esa cifra en S→XL, así que debe escalar, no ser plano.</t>
+          <t>La fila ahora se lee en una sola pasada: base (construyo) → feedback (valido) → total en días → total en monedas — con fórmula, sin sacar la cuenta por fuera. Antes las monedas salían del día BASE (a mitad de la fila) en vez del total con feedback.</t>
         </is>
       </c>
       <c r="E6" s="2" t="n"/>
@@ -882,17 +882,17 @@
       <c r="C7" s="2" t="n"/>
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="3" t="n"/>
-      <c r="F7" s="11" t="inlineStr">
-        <is>
-          <t>Monedas 🪙 equivalentes</t>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Feedback + VB (días extra por talla)</t>
         </is>
       </c>
       <c r="G7" s="2" t="n"/>
       <c r="H7" s="2" t="n"/>
       <c r="I7" s="3" t="n"/>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>Feedback + VB (días extra por talla)</t>
+      <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>Appetite total (días, base + feedback)</t>
         </is>
       </c>
       <c r="K7" s="2" t="n"/>
@@ -900,7 +900,7 @@
       <c r="M7" s="3" t="n"/>
       <c r="N7" s="12" t="inlineStr">
         <is>
-          <t>Appetite total con feedback (días)</t>
+          <t>Monedas 🪙 (total con feedback)</t>
         </is>
       </c>
       <c r="O7" s="2" t="n"/>
@@ -937,42 +937,42 @@
           <t>XL</t>
         </is>
       </c>
-      <c r="F8" s="11" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="G8" s="11" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="H8" s="11" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="I8" s="11" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>XL</t>
         </is>
       </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="J8" s="11" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="K8" s="6" t="inlineStr">
+      <c r="K8" s="11" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="L8" s="6" t="inlineStr">
+      <c r="L8" s="11" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="M8" s="6" t="inlineStr">
+      <c r="M8" s="11" t="inlineStr">
         <is>
           <t>XL</t>
         </is>
@@ -1035,64 +1035,64 @@
           <t>Programa completo de punta a punta, multicanal (p. ej. ecosistema de entendimiento)</t>
         </is>
       </c>
-      <c r="F9" s="17" t="inlineStr">
-        <is>
-          <t>días × 0.72</t>
-        </is>
-      </c>
-      <c r="G9" s="17" t="inlineStr">
-        <is>
-          <t>días × 0.72</t>
-        </is>
-      </c>
-      <c r="H9" s="17" t="inlineStr">
-        <is>
-          <t>días × 0.72</t>
-        </is>
-      </c>
-      <c r="I9" s="17" t="inlineStr">
-        <is>
-          <t>días × 0.72</t>
-        </is>
-      </c>
-      <c r="J9" s="16" t="inlineStr">
+      <c r="F9" s="16" t="inlineStr">
         <is>
           <t>0–1d: sin gate, o 1 revisor rápido (&lt;48h)</t>
         </is>
       </c>
-      <c r="K9" s="16" t="inlineStr">
+      <c r="G9" s="16" t="inlineStr">
         <is>
           <t>1–2d: feedback estándar de 1 stakeholder</t>
         </is>
       </c>
-      <c r="L9" s="16" t="inlineStr">
+      <c r="H9" s="16" t="inlineStr">
         <is>
           <t>2d: 1 gate externo (comité o revisión formal)</t>
         </is>
       </c>
-      <c r="M9" s="16" t="inlineStr">
+      <c r="I9" s="16" t="inlineStr">
         <is>
           <t>3d+: 2+ gates (legal, médico, comité)</t>
         </is>
       </c>
+      <c r="J9" s="17" t="inlineStr">
+        <is>
+          <t>Base + Feedback</t>
+        </is>
+      </c>
+      <c r="K9" s="17" t="inlineStr">
+        <is>
+          <t>Base + Feedback</t>
+        </is>
+      </c>
+      <c r="L9" s="17" t="inlineStr">
+        <is>
+          <t>Base + Feedback</t>
+        </is>
+      </c>
+      <c r="M9" s="17" t="inlineStr">
+        <is>
+          <t>Base + Feedback</t>
+        </is>
+      </c>
       <c r="N9" s="18" t="inlineStr">
         <is>
-          <t>ANS Base + Feedback</t>
+          <t>total × 0.72</t>
         </is>
       </c>
       <c r="O9" s="18" t="inlineStr">
         <is>
-          <t>ANS Base + Feedback</t>
+          <t>total × 0.72</t>
         </is>
       </c>
       <c r="P9" s="18" t="inlineStr">
         <is>
-          <t>ANS Base + Feedback</t>
+          <t>total × 0.72</t>
         </is>
       </c>
       <c r="Q9" s="18" t="inlineStr">
         <is>
-          <t>ANS Base + Feedback</t>
+          <t>total × 0.72</t>
         </is>
       </c>
       <c r="R9" s="19" t="inlineStr">
@@ -1130,48 +1130,48 @@
       <c r="E10" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="F10" s="22">
-        <f>B10*$F$4</f>
-        <v/>
-      </c>
-      <c r="G10" s="22">
-        <f>C10*$F$4</f>
-        <v/>
-      </c>
-      <c r="H10" s="22">
-        <f>D10*$F$4</f>
-        <v/>
-      </c>
-      <c r="I10" s="22">
-        <f>E10*$F$4</f>
-        <v/>
-      </c>
-      <c r="J10" s="21" t="n">
+      <c r="F10" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="21" t="n">
+      <c r="G10" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="L10" s="21" t="n">
+      <c r="H10" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="M10" s="21" t="n">
+      <c r="I10" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="N10" s="21">
-        <f>B10+J10</f>
-        <v/>
-      </c>
-      <c r="O10" s="21">
-        <f>C10+K10</f>
-        <v/>
-      </c>
-      <c r="P10" s="21">
-        <f>D10+L10</f>
-        <v/>
-      </c>
-      <c r="Q10" s="21">
-        <f>E10+M10</f>
+      <c r="J10" s="21">
+        <f>B10+F10</f>
+        <v/>
+      </c>
+      <c r="K10" s="21">
+        <f>C10+G10</f>
+        <v/>
+      </c>
+      <c r="L10" s="21">
+        <f>D10+H10</f>
+        <v/>
+      </c>
+      <c r="M10" s="21">
+        <f>E10+I10</f>
+        <v/>
+      </c>
+      <c r="N10" s="22">
+        <f>J10*$F$4</f>
+        <v/>
+      </c>
+      <c r="O10" s="22">
+        <f>K10*$F$4</f>
+        <v/>
+      </c>
+      <c r="P10" s="22">
+        <f>L10*$F$4</f>
+        <v/>
+      </c>
+      <c r="Q10" s="22">
+        <f>M10*$F$4</f>
         <v/>
       </c>
     </row>
@@ -1194,48 +1194,48 @@
       <c r="E11" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="F11" s="22">
-        <f>B11*$F$4</f>
-        <v/>
-      </c>
-      <c r="G11" s="22">
-        <f>C11*$F$4</f>
-        <v/>
-      </c>
-      <c r="H11" s="22">
-        <f>D11*$F$4</f>
-        <v/>
-      </c>
-      <c r="I11" s="22">
-        <f>E11*$F$4</f>
-        <v/>
-      </c>
-      <c r="J11" s="21" t="n">
+      <c r="F11" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="21" t="n">
+      <c r="G11" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="L11" s="21" t="n">
+      <c r="H11" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="M11" s="21" t="n">
+      <c r="I11" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="N11" s="21">
-        <f>B11+J11</f>
-        <v/>
-      </c>
-      <c r="O11" s="21">
-        <f>C11+K11</f>
-        <v/>
-      </c>
-      <c r="P11" s="21">
-        <f>D11+L11</f>
-        <v/>
-      </c>
-      <c r="Q11" s="21">
-        <f>E11+M11</f>
+      <c r="J11" s="21">
+        <f>B11+F11</f>
+        <v/>
+      </c>
+      <c r="K11" s="21">
+        <f>C11+G11</f>
+        <v/>
+      </c>
+      <c r="L11" s="21">
+        <f>D11+H11</f>
+        <v/>
+      </c>
+      <c r="M11" s="21">
+        <f>E11+I11</f>
+        <v/>
+      </c>
+      <c r="N11" s="22">
+        <f>J11*$F$4</f>
+        <v/>
+      </c>
+      <c r="O11" s="22">
+        <f>K11*$F$4</f>
+        <v/>
+      </c>
+      <c r="P11" s="22">
+        <f>L11*$F$4</f>
+        <v/>
+      </c>
+      <c r="Q11" s="22">
+        <f>M11*$F$4</f>
         <v/>
       </c>
     </row>
@@ -1258,48 +1258,48 @@
       <c r="E12" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="F12" s="22">
-        <f>B12*$F$4</f>
-        <v/>
-      </c>
-      <c r="G12" s="22">
-        <f>C12*$F$4</f>
-        <v/>
-      </c>
-      <c r="H12" s="22">
-        <f>D12*$F$4</f>
-        <v/>
-      </c>
-      <c r="I12" s="22">
-        <f>E12*$F$4</f>
-        <v/>
-      </c>
-      <c r="J12" s="21" t="n">
+      <c r="F12" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="K12" s="21" t="n">
+      <c r="G12" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="L12" s="21" t="n">
+      <c r="H12" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="M12" s="21" t="n">
+      <c r="I12" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="N12" s="21">
-        <f>B12+J12</f>
-        <v/>
-      </c>
-      <c r="O12" s="21">
-        <f>C12+K12</f>
-        <v/>
-      </c>
-      <c r="P12" s="21">
-        <f>D12+L12</f>
-        <v/>
-      </c>
-      <c r="Q12" s="21">
-        <f>E12+M12</f>
+      <c r="J12" s="21">
+        <f>B12+F12</f>
+        <v/>
+      </c>
+      <c r="K12" s="21">
+        <f>C12+G12</f>
+        <v/>
+      </c>
+      <c r="L12" s="21">
+        <f>D12+H12</f>
+        <v/>
+      </c>
+      <c r="M12" s="21">
+        <f>E12+I12</f>
+        <v/>
+      </c>
+      <c r="N12" s="22">
+        <f>J12*$F$4</f>
+        <v/>
+      </c>
+      <c r="O12" s="22">
+        <f>K12*$F$4</f>
+        <v/>
+      </c>
+      <c r="P12" s="22">
+        <f>L12*$F$4</f>
+        <v/>
+      </c>
+      <c r="Q12" s="22">
+        <f>M12*$F$4</f>
         <v/>
       </c>
     </row>
@@ -1322,48 +1322,48 @@
       <c r="E13" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="F13" s="22">
-        <f>B13*$F$4</f>
-        <v/>
-      </c>
-      <c r="G13" s="22">
-        <f>C13*$F$4</f>
-        <v/>
-      </c>
-      <c r="H13" s="22">
-        <f>D13*$F$4</f>
-        <v/>
-      </c>
-      <c r="I13" s="22">
-        <f>E13*$F$4</f>
-        <v/>
-      </c>
-      <c r="J13" s="21" t="n">
+      <c r="F13" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="21" t="n">
+      <c r="G13" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="L13" s="21" t="n">
+      <c r="H13" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="M13" s="21" t="n">
+      <c r="I13" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="N13" s="21">
-        <f>B13+J13</f>
-        <v/>
-      </c>
-      <c r="O13" s="21">
-        <f>C13+K13</f>
-        <v/>
-      </c>
-      <c r="P13" s="21">
-        <f>D13+L13</f>
-        <v/>
-      </c>
-      <c r="Q13" s="21">
-        <f>E13+M13</f>
+      <c r="J13" s="21">
+        <f>B13+F13</f>
+        <v/>
+      </c>
+      <c r="K13" s="21">
+        <f>C13+G13</f>
+        <v/>
+      </c>
+      <c r="L13" s="21">
+        <f>D13+H13</f>
+        <v/>
+      </c>
+      <c r="M13" s="21">
+        <f>E13+I13</f>
+        <v/>
+      </c>
+      <c r="N13" s="22">
+        <f>J13*$F$4</f>
+        <v/>
+      </c>
+      <c r="O13" s="22">
+        <f>K13*$F$4</f>
+        <v/>
+      </c>
+      <c r="P13" s="22">
+        <f>L13*$F$4</f>
+        <v/>
+      </c>
+      <c r="Q13" s="22">
+        <f>M13*$F$4</f>
         <v/>
       </c>
     </row>
@@ -1386,48 +1386,48 @@
       <c r="E14" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="F14" s="22">
-        <f>B14*$F$4</f>
-        <v/>
-      </c>
-      <c r="G14" s="22">
-        <f>C14*$F$4</f>
-        <v/>
-      </c>
-      <c r="H14" s="22">
-        <f>D14*$F$4</f>
-        <v/>
-      </c>
-      <c r="I14" s="22">
-        <f>E14*$F$4</f>
-        <v/>
-      </c>
-      <c r="J14" s="21" t="n">
+      <c r="F14" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="K14" s="21" t="n">
+      <c r="G14" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="L14" s="21" t="n">
+      <c r="H14" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="M14" s="21" t="n">
+      <c r="I14" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="N14" s="21">
-        <f>B14+J14</f>
-        <v/>
-      </c>
-      <c r="O14" s="21">
-        <f>C14+K14</f>
-        <v/>
-      </c>
-      <c r="P14" s="21">
-        <f>D14+L14</f>
-        <v/>
-      </c>
-      <c r="Q14" s="21">
-        <f>E14+M14</f>
+      <c r="J14" s="21">
+        <f>B14+F14</f>
+        <v/>
+      </c>
+      <c r="K14" s="21">
+        <f>C14+G14</f>
+        <v/>
+      </c>
+      <c r="L14" s="21">
+        <f>D14+H14</f>
+        <v/>
+      </c>
+      <c r="M14" s="21">
+        <f>E14+I14</f>
+        <v/>
+      </c>
+      <c r="N14" s="22">
+        <f>J14*$F$4</f>
+        <v/>
+      </c>
+      <c r="O14" s="22">
+        <f>K14*$F$4</f>
+        <v/>
+      </c>
+      <c r="P14" s="22">
+        <f>L14*$F$4</f>
+        <v/>
+      </c>
+      <c r="Q14" s="22">
+        <f>M14*$F$4</f>
         <v/>
       </c>
     </row>
@@ -1450,48 +1450,48 @@
       <c r="E15" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="F15" s="22">
-        <f>B15*$F$4</f>
-        <v/>
-      </c>
-      <c r="G15" s="22">
-        <f>C15*$F$4</f>
-        <v/>
-      </c>
-      <c r="H15" s="22">
-        <f>D15*$F$4</f>
-        <v/>
-      </c>
-      <c r="I15" s="22">
-        <f>E15*$F$4</f>
-        <v/>
-      </c>
-      <c r="J15" s="21" t="n">
+      <c r="F15" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="K15" s="21" t="n">
+      <c r="G15" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="L15" s="21" t="n">
+      <c r="H15" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="M15" s="21" t="n">
+      <c r="I15" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="N15" s="21">
-        <f>B15+J15</f>
-        <v/>
-      </c>
-      <c r="O15" s="21">
-        <f>C15+K15</f>
-        <v/>
-      </c>
-      <c r="P15" s="21">
-        <f>D15+L15</f>
-        <v/>
-      </c>
-      <c r="Q15" s="21">
-        <f>E15+M15</f>
+      <c r="J15" s="21">
+        <f>B15+F15</f>
+        <v/>
+      </c>
+      <c r="K15" s="21">
+        <f>C15+G15</f>
+        <v/>
+      </c>
+      <c r="L15" s="21">
+        <f>D15+H15</f>
+        <v/>
+      </c>
+      <c r="M15" s="21">
+        <f>E15+I15</f>
+        <v/>
+      </c>
+      <c r="N15" s="22">
+        <f>J15*$F$4</f>
+        <v/>
+      </c>
+      <c r="O15" s="22">
+        <f>K15*$F$4</f>
+        <v/>
+      </c>
+      <c r="P15" s="22">
+        <f>L15*$F$4</f>
+        <v/>
+      </c>
+      <c r="Q15" s="22">
+        <f>M15*$F$4</f>
         <v/>
       </c>
     </row>
@@ -1548,64 +1548,64 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F17" s="24" t="inlineStr">
+      <c r="F17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N17" s="24" t="inlineStr">
         <is>
           <t>1–2 🪙/trim.</t>
         </is>
       </c>
-      <c r="G17" s="24" t="inlineStr">
+      <c r="O17" s="24" t="inlineStr">
         <is>
           <t>3–4 🪙/trim.</t>
         </is>
       </c>
-      <c r="H17" s="24" t="inlineStr">
+      <c r="P17" s="24" t="inlineStr">
         <is>
           <t>5–6 🪙/trim.</t>
         </is>
       </c>
-      <c r="I17" s="24" t="inlineStr">
+      <c r="Q17" s="24" t="inlineStr">
         <is>
           <t>7–8 🪙/trim.</t>
-        </is>
-      </c>
-      <c r="J17" s="21" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="K17" s="21" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="L17" s="21" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="M17" s="21" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="N17" s="21" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="O17" s="21" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="P17" s="21" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="Q17" s="21" t="inlineStr">
-        <is>
-          <t>NA</t>
         </is>
       </c>
       <c r="R17" s="25" t="inlineStr">

</xml_diff>